<commit_message>
Add demo vitals and encounter identifier system
</commit_message>
<xml_diff>
--- a/FHIR_Testdatengenerator_Interpolar_Demo.xlsx
+++ b/FHIR_Testdatengenerator_Interpolar_Demo.xlsx
@@ -35,8 +35,8 @@
     <numFmt numFmtId="167" formatCode="dd/mm/yyyy\ hh:mm;@"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="00000000"/>
-    <numFmt numFmtId="170" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="171" formatCode="dd.mm.yyyy hh:mm:ss"/>
+    <numFmt numFmtId="170" formatCode="dd.mm.yyyy hh:mm:ss"/>
+    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -254,7 +254,7 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -430,11 +430,11 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -493,6 +493,11 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -878,120 +883,120 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="58">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="52" t="inlineStr">
         <is>
           <t>Paula</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="52" t="inlineStr">
         <is>
           <t>Positiveins</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="52" t="inlineStr">
         <is>
           <t>Demoallee 1, 53121 Bonn</t>
         </is>
       </c>
-      <c r="E2" s="59" t="n">
+      <c r="E2" s="82" t="n">
         <v>18264</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="52" t="inlineStr">
         <is>
           <t>weiblich</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="52" t="inlineStr">
         <is>
           <t>AOK</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="52" t="inlineStr">
         <is>
           <t>Demo-Patient mit zwei erwarteten MRP-Triggern.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="58">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="52" t="inlineStr">
         <is>
           <t>Bernd</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="52" t="inlineStr">
         <is>
           <t>Lebermann</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="52" t="inlineStr">
         <is>
           <t>Demoallee 2, 53121 Bonn</t>
         </is>
       </c>
-      <c r="E3" s="59" t="n">
+      <c r="E3" s="82" t="n">
         <v>20090</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="52" t="inlineStr">
         <is>
           <t>männlich</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="52" t="inlineStr">
         <is>
           <t>Techniker</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="52" t="inlineStr">
         <is>
           <t>Demo-Patient mit einem erwarteten MRP-Trigger.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="58">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="52" t="inlineStr">
         <is>
           <t>Clara</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="52" t="inlineStr">
         <is>
           <t>Kontrolle</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="52" t="inlineStr">
         <is>
           <t>Demoallee 3, 53121 Bonn</t>
         </is>
       </c>
-      <c r="E4" s="59" t="n">
+      <c r="E4" s="82" t="n">
         <v>21916</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="52" t="inlineStr">
         <is>
           <t>weiblich</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="52" t="inlineStr">
         <is>
           <t>AOK plus</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N4" s="52" t="inlineStr">
         <is>
           <t>In-progress-Kontrollpatient ohne erwartetes MRP.</t>
         </is>
@@ -2580,190 +2585,190 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="58">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00001</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="59" t="n">
+      <c r="C2" s="82" t="n">
         <v>46143.33333333334</v>
       </c>
-      <c r="D2" s="59" t="n">
+      <c r="D2" s="82" t="n">
         <v>46147.5</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="52" t="inlineStr">
         <is>
           <t>stationaer</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="52" t="inlineStr">
         <is>
           <t>Innere Medizin</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="52" t="inlineStr">
         <is>
           <t>INTERPOLAR-01</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="52" t="inlineStr">
         <is>
           <t>R101</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="52" t="inlineStr">
         <is>
           <t>Erster Versorgungsstellenkontakt; Tag-3-Daten liegen hier.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="58">
-      <c r="C3" s="59" t="n">
+      <c r="C3" s="82" t="n">
         <v>46147.5</v>
       </c>
-      <c r="D3" s="59" t="n">
+      <c r="D3" s="82" t="n">
         <v>46152.5</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="52" t="inlineStr">
         <is>
           <t>INTERPOLAR-01</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="52" t="inlineStr">
         <is>
           <t>R102</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="52" t="inlineStr">
         <is>
           <t>Gleicher Abteilungskontakt, zweiter Versorgungsstellenkontakt.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="58">
-      <c r="C4" s="59" t="n">
+      <c r="C4" s="82" t="n">
         <v>46152.5</v>
       </c>
-      <c r="D4" s="59" t="n">
+      <c r="D4" s="82" t="n">
         <v>46157.5</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="52" t="inlineStr">
         <is>
           <t>INTERPOLAR-02</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="52" t="inlineStr">
         <is>
           <t>R201</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="52" t="inlineStr">
         <is>
           <t>Gleicher Abteilungskontakt, dritter Versorgungsstellenkontakt.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="58">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00002</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="59" t="n">
+      <c r="C5" s="82" t="n">
         <v>46143.375</v>
       </c>
-      <c r="D5" s="59" t="n">
+      <c r="D5" s="82" t="n">
         <v>46150.5</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="52" t="inlineStr">
         <is>
           <t>stationaer</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="52" t="inlineStr">
         <is>
           <t>Innere Medizin</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="52" t="inlineStr">
         <is>
           <t>INTERPOLAR-02</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="52" t="inlineStr">
         <is>
           <t>R202</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="52" t="inlineStr">
         <is>
           <t>Erster Versorgungsstellenkontakt; Tag-3-Daten liegen hier.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="58">
-      <c r="C6" s="59" t="n">
+      <c r="C6" s="82" t="n">
         <v>46150.5</v>
       </c>
-      <c r="D6" s="59" t="n">
+      <c r="D6" s="82" t="n">
         <v>46157.5</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="52" t="inlineStr">
         <is>
           <t>INTERPOLAR-02</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="52" t="inlineStr">
         <is>
           <t>R203</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="52" t="inlineStr">
         <is>
           <t>Gleicher Abteilungskontakt, zweiter Versorgungsstellenkontakt.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="58">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00003</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="59" t="n">
+      <c r="C7" s="82" t="n">
         <v>46143.41666666666</v>
       </c>
-      <c r="D7" s="61" t="n"/>
-      <c r="E7" t="inlineStr">
+      <c r="D7" s="83" t="n"/>
+      <c r="E7" s="52" t="inlineStr">
         <is>
           <t>stationaer</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="52" t="inlineStr">
         <is>
           <t>Innere Medizin</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="52" t="inlineStr">
         <is>
           <t>INTERPOLAR-03</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="52" t="inlineStr">
         <is>
           <t>R301</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="52" t="inlineStr">
         <is>
           <t>In-progress-Kontakt ohne Ende.</t>
         </is>
@@ -2875,72 +2880,72 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="58">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00001</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="52" t="inlineStr">
         <is>
           <t>2951-2</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="52" t="inlineStr">
         <is>
           <t>Natrium</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="52" t="n">
         <v>60</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="52" t="inlineStr">
         <is>
           <t>umol/L</t>
         </is>
       </c>
-      <c r="G2" s="59" t="n">
+      <c r="G2" s="82" t="n">
         <v>46145.41666666666</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="52" t="inlineStr">
         <is>
           <t>Tag 3 nach Aufnahme, innerhalb des ersten Versorgungsstellenkontakts.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="58">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00002</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="52" t="inlineStr">
         <is>
           <t>1751-7</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="52" t="inlineStr">
         <is>
           <t>Albumin</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="52" t="n">
         <v>10</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="52" t="inlineStr">
         <is>
           <t>g/L</t>
         </is>
       </c>
-      <c r="G3" s="59" t="n">
+      <c r="G3" s="82" t="n">
         <v>46145.41666666666</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="52" t="inlineStr">
         <is>
           <t>Tag 3 nach Aufnahme, innerhalb des ersten Versorgungsstellenkontakts.</t>
         </is>
@@ -3598,66 +3603,66 @@
       <c r="J1" s="64" t="n"/>
     </row>
     <row r="2" ht="15" customFormat="1" customHeight="1" s="55">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00001</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="52" t="inlineStr">
         <is>
           <t>Hypokaliämie</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="52" t="inlineStr">
         <is>
           <t>E87.6</t>
         </is>
       </c>
-      <c r="E2" s="59" t="n">
+      <c r="E2" s="82" t="n">
         <v>46145.4375</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="52" t="inlineStr">
         <is>
           <t>Nebendiagnose</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="52" t="inlineStr">
         <is>
           <t>Tag 3 nach Aufnahme, innerhalb des ersten Versorgungsstellenkontakts.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customFormat="1" customHeight="1" s="55">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00003</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="52" t="inlineStr">
         <is>
           <t>Vorher bestehende Hypertonie in der Schwangerschaft</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="52" t="inlineStr">
         <is>
           <t>O10</t>
         </is>
       </c>
-      <c r="E3" s="59" t="n">
+      <c r="E3" s="82" t="n">
         <v>46145.4375</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="52" t="inlineStr">
         <is>
           <t>Nebendiagnose</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="52" t="inlineStr">
         <is>
           <t>Kontrolltrigger, aber Fall ist noch nicht beendet.</t>
         </is>
@@ -4052,258 +4057,258 @@
       </c>
     </row>
     <row r="2" ht="15" customFormat="1" customHeight="1" s="55">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00001</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="59" t="n">
+      <c r="C2" s="82" t="n">
         <v>46145.375</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="52" t="inlineStr">
         <is>
           <t>Verordnung (MedicationRequest)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="52" t="inlineStr">
         <is>
           <t>Am Aufnahmetag</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="52" t="inlineStr">
         <is>
           <t>Demo S01EC01</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="52" t="inlineStr">
         <is>
           <t>S01EC01</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="52" t="inlineStr">
         <is>
           <t>ATC</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="52" t="inlineStr">
         <is>
           <t>Tabletten</t>
         </is>
       </c>
-      <c r="L2" s="59" t="n">
+      <c r="L2" s="82" t="n">
         <v>46145.375</v>
       </c>
-      <c r="M2" s="59" t="n">
+      <c r="M2" s="82" t="n">
         <v>46157.5</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="52" t="inlineStr">
         <is>
           <t>mg</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="P2" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" s="52" t="inlineStr">
         <is>
           <t>MRP-Demo-Medikation.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customFormat="1" customHeight="1" s="55">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00001</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="59" t="n">
+      <c r="C3" s="82" t="n">
         <v>46145.375</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="52" t="inlineStr">
         <is>
           <t>Verordnung (MedicationRequest)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="52" t="inlineStr">
         <is>
           <t>Am Aufnahmetag</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="52" t="inlineStr">
         <is>
           <t>Demo S01EC02</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="52" t="inlineStr">
         <is>
           <t>S01EC02</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="52" t="inlineStr">
         <is>
           <t>ATC</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="52" t="inlineStr">
         <is>
           <t>Tabletten</t>
         </is>
       </c>
-      <c r="L3" s="59" t="n">
+      <c r="L3" s="82" t="n">
         <v>46145.375</v>
       </c>
-      <c r="M3" s="59" t="n">
+      <c r="M3" s="82" t="n">
         <v>46157.5</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="52" t="inlineStr">
         <is>
           <t>mg</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="P3" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q3" s="52" t="inlineStr">
         <is>
           <t>MRP-Demo-Medikation.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customFormat="1" customHeight="1" s="55">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00002</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="59" t="n">
+      <c r="C4" s="82" t="n">
         <v>46145.375</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="52" t="inlineStr">
         <is>
           <t>Verordnung (MedicationRequest)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="52" t="inlineStr">
         <is>
           <t>Am Aufnahmetag</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="52" t="inlineStr">
         <is>
           <t>Demo L01XK52</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="52" t="inlineStr">
         <is>
           <t>L01XK52</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="52" t="inlineStr">
         <is>
           <t>ATC</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="52" t="inlineStr">
         <is>
           <t>Tabletten</t>
         </is>
       </c>
-      <c r="L4" s="59" t="n">
+      <c r="L4" s="82" t="n">
         <v>46145.375</v>
       </c>
-      <c r="M4" s="59" t="n">
+      <c r="M4" s="82" t="n">
         <v>46157.5</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="52" t="inlineStr">
         <is>
           <t>mg</t>
         </is>
       </c>
-      <c r="P4" t="n">
+      <c r="P4" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q4" s="52" t="inlineStr">
         <is>
           <t>MRP-Demo-Medikation.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customFormat="1" customHeight="1" s="55">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="52" t="inlineStr">
         <is>
           <t>Interpolar_Demo_Patient_00003</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="59" t="n">
+      <c r="C5" s="82" t="n">
         <v>46145.375</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="52" t="inlineStr">
         <is>
           <t>Verordnung (MedicationRequest)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="52" t="inlineStr">
         <is>
           <t>Am Aufnahmetag</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="52" t="inlineStr">
         <is>
           <t>Demo M01AB11</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="52" t="inlineStr">
         <is>
           <t>M01AB11</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="52" t="inlineStr">
         <is>
           <t>ATC</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="52" t="inlineStr">
         <is>
           <t>Tabletten</t>
         </is>
       </c>
-      <c r="L5" s="59" t="n">
+      <c r="L5" s="82" t="n">
         <v>46145.375</v>
       </c>
-      <c r="M5" s="61" t="n"/>
-      <c r="N5" t="n">
+      <c r="M5" s="83" t="n"/>
+      <c r="N5" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="52" t="inlineStr">
         <is>
           <t>mg</t>
         </is>
       </c>
-      <c r="P5" t="n">
+      <c r="P5" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q5" s="52" t="inlineStr">
         <is>
           <t>Kontrollmedikation, aber Fall ist noch nicht beendet.</t>
         </is>
@@ -4494,13 +4499,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24.29" customWidth="1" style="62" min="1" max="1"/>
     <col width="7" customWidth="1" style="52" min="2" max="2"/>
     <col width="28.86" customWidth="1" style="62" min="3" max="3"/>
     <col width="8.710000000000001" customWidth="1" style="62" min="4" max="6"/>
+    <col width="13" customWidth="1" style="58" min="5" max="5"/>
+    <col width="13" customWidth="1" style="58" min="6" max="6"/>
     <col width="23" customWidth="1" style="66" min="7" max="7"/>
     <col width="29.42" customWidth="1" style="62" min="8" max="8"/>
     <col width="9.710000000000001" customWidth="1" style="62" min="9" max="9"/>
@@ -4549,12 +4556,198 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="58"/>
-    <row r="3" ht="15" customHeight="1" s="58"/>
-    <row r="4" ht="15" customHeight="1" s="58"/>
-    <row r="5" ht="15" customHeight="1" s="58"/>
-    <row r="6" ht="15" customHeight="1" s="58"/>
-    <row r="7" ht="15" customHeight="1" s="58"/>
+    <row r="2" ht="15" customHeight="1" s="58">
+      <c r="A2" s="62" t="inlineStr">
+        <is>
+          <t>Interpolar_Demo_Patient_00001</t>
+        </is>
+      </c>
+      <c r="B2" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="62" t="inlineStr">
+        <is>
+          <t>Körpergewicht</t>
+        </is>
+      </c>
+      <c r="D2" s="62" t="inlineStr">
+        <is>
+          <t>3142-7</t>
+        </is>
+      </c>
+      <c r="E2" s="62" t="n">
+        <v>82</v>
+      </c>
+      <c r="F2" s="62" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G2" s="84" t="n">
+        <v>46145.35416666666</v>
+      </c>
+      <c r="H2" s="54" t="n"/>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="58">
+      <c r="A3" s="62" t="inlineStr">
+        <is>
+          <t>Interpolar_Demo_Patient_00001</t>
+        </is>
+      </c>
+      <c r="B3" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="62" t="inlineStr">
+        <is>
+          <t>Körpergröße</t>
+        </is>
+      </c>
+      <c r="D3" s="62" t="inlineStr">
+        <is>
+          <t>8302-2</t>
+        </is>
+      </c>
+      <c r="E3" s="62" t="n">
+        <v>176</v>
+      </c>
+      <c r="F3" s="62" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="G3" s="84" t="n">
+        <v>46145.35763888889</v>
+      </c>
+      <c r="H3" s="54" t="n"/>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="58">
+      <c r="A4" s="62" t="inlineStr">
+        <is>
+          <t>Interpolar_Demo_Patient_00002</t>
+        </is>
+      </c>
+      <c r="B4" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>Körpergewicht</t>
+        </is>
+      </c>
+      <c r="D4" s="62" t="inlineStr">
+        <is>
+          <t>3142-7</t>
+        </is>
+      </c>
+      <c r="E4" s="62" t="n">
+        <v>74</v>
+      </c>
+      <c r="F4" s="62" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G4" s="84" t="n">
+        <v>46145.35416666666</v>
+      </c>
+      <c r="H4" s="54" t="n"/>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="58">
+      <c r="A5" s="62" t="inlineStr">
+        <is>
+          <t>Interpolar_Demo_Patient_00002</t>
+        </is>
+      </c>
+      <c r="B5" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="62" t="inlineStr">
+        <is>
+          <t>Körpergröße</t>
+        </is>
+      </c>
+      <c r="D5" s="62" t="inlineStr">
+        <is>
+          <t>8302-2</t>
+        </is>
+      </c>
+      <c r="E5" s="62" t="n">
+        <v>180</v>
+      </c>
+      <c r="F5" s="62" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="G5" s="84" t="n">
+        <v>46145.35763888889</v>
+      </c>
+      <c r="H5" s="54" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="58">
+      <c r="A6" s="62" t="inlineStr">
+        <is>
+          <t>Interpolar_Demo_Patient_00003</t>
+        </is>
+      </c>
+      <c r="B6" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="62" t="inlineStr">
+        <is>
+          <t>Körpergewicht</t>
+        </is>
+      </c>
+      <c r="D6" s="62" t="inlineStr">
+        <is>
+          <t>3142-7</t>
+        </is>
+      </c>
+      <c r="E6" s="62" t="n">
+        <v>68</v>
+      </c>
+      <c r="F6" s="62" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G6" s="84" t="n">
+        <v>46145.35416666666</v>
+      </c>
+      <c r="H6" s="54" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="58">
+      <c r="A7" s="62" t="inlineStr">
+        <is>
+          <t>Interpolar_Demo_Patient_00003</t>
+        </is>
+      </c>
+      <c r="B7" s="52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="62" t="inlineStr">
+        <is>
+          <t>Körpergröße</t>
+        </is>
+      </c>
+      <c r="D7" s="62" t="inlineStr">
+        <is>
+          <t>8302-2</t>
+        </is>
+      </c>
+      <c r="E7" s="62" t="n">
+        <v>168</v>
+      </c>
+      <c r="F7" s="62" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="G7" s="84" t="n">
+        <v>46145.35763888889</v>
+      </c>
+      <c r="H7" s="54" t="n"/>
+    </row>
     <row r="8" ht="15" customHeight="1" s="58"/>
     <row r="9" ht="15" customHeight="1" s="58"/>
     <row r="10" ht="15" customHeight="1" s="58"/>

</xml_diff>

<commit_message>
Shift Interpolar demo dates to April
</commit_message>
<xml_diff>
--- a/FHIR_Testdatengenerator_Interpolar_Demo.xlsx
+++ b/FHIR_Testdatengenerator_Interpolar_Demo.xlsx
@@ -904,7 +904,7 @@
         </is>
       </c>
       <c r="E2" s="82" t="n">
-        <v>18264</v>
+        <v>18233</v>
       </c>
       <c r="F2" s="52" t="inlineStr">
         <is>
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="E3" s="82" t="n">
-        <v>20090</v>
+        <v>20059</v>
       </c>
       <c r="F3" s="52" t="inlineStr">
         <is>
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="E4" s="82" t="n">
-        <v>21916</v>
+        <v>21885</v>
       </c>
       <c r="F4" s="52" t="inlineStr">
         <is>
@@ -1853,6 +1853,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="58">
       <c r="A50" s="78" t="inlineStr">
         <is>
@@ -1909,6 +1910,7 @@
         </is>
       </c>
     </row>
+    <row r="58"/>
     <row r="59" ht="15" customHeight="1" s="58">
       <c r="A59" s="78" t="inlineStr">
         <is>
@@ -1951,6 +1953,8 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
+    <row r="66"/>
     <row r="67" ht="15" customHeight="1" s="58">
       <c r="A67" s="78" t="inlineStr">
         <is>
@@ -2049,6 +2053,7 @@
         </is>
       </c>
     </row>
+    <row r="81"/>
     <row r="82" ht="15" customHeight="1" s="58">
       <c r="A82" s="78" t="inlineStr">
         <is>
@@ -2140,6 +2145,8 @@
         </is>
       </c>
     </row>
+    <row r="95"/>
+    <row r="96"/>
     <row r="97" ht="15" customHeight="1" s="58">
       <c r="A97" s="78" t="inlineStr">
         <is>
@@ -2238,6 +2245,7 @@
         </is>
       </c>
     </row>
+    <row r="111"/>
     <row r="112" ht="15" customHeight="1" s="58">
       <c r="A112" s="78" t="inlineStr">
         <is>
@@ -2329,6 +2337,8 @@
         </is>
       </c>
     </row>
+    <row r="125"/>
+    <row r="126"/>
     <row r="127" ht="15" customHeight="1" s="58">
       <c r="A127" s="78" t="inlineStr">
         <is>
@@ -2413,6 +2423,8 @@
         </is>
       </c>
     </row>
+    <row r="139"/>
+    <row r="140"/>
     <row r="141" ht="15" customHeight="1" s="58">
       <c r="A141" s="78" t="inlineStr">
         <is>
@@ -2490,6 +2502,7 @@
         </is>
       </c>
     </row>
+    <row r="152"/>
     <row r="153" ht="15" customHeight="1" s="58">
       <c r="A153" s="78" t="inlineStr">
         <is>
@@ -2594,10 +2607,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="82" t="n">
-        <v>46143.33333333334</v>
+        <v>46113.33333333334</v>
       </c>
       <c r="D2" s="82" t="n">
-        <v>46147.5</v>
+        <v>46117.5</v>
       </c>
       <c r="E2" s="52" t="inlineStr">
         <is>
@@ -2627,10 +2640,10 @@
     </row>
     <row r="3" ht="15" customHeight="1" s="58">
       <c r="C3" s="82" t="n">
-        <v>46147.5</v>
+        <v>46117.5</v>
       </c>
       <c r="D3" s="82" t="n">
-        <v>46152.5</v>
+        <v>46122.5</v>
       </c>
       <c r="G3" s="52" t="inlineStr">
         <is>
@@ -2650,10 +2663,10 @@
     </row>
     <row r="4" ht="15" customHeight="1" s="58">
       <c r="C4" s="82" t="n">
-        <v>46152.5</v>
+        <v>46122.5</v>
       </c>
       <c r="D4" s="82" t="n">
-        <v>46157.5</v>
+        <v>46127.5</v>
       </c>
       <c r="G4" s="52" t="inlineStr">
         <is>
@@ -2681,10 +2694,10 @@
         <v>1</v>
       </c>
       <c r="C5" s="82" t="n">
-        <v>46143.375</v>
+        <v>46113.375</v>
       </c>
       <c r="D5" s="82" t="n">
-        <v>46150.5</v>
+        <v>46120.5</v>
       </c>
       <c r="E5" s="52" t="inlineStr">
         <is>
@@ -2714,10 +2727,10 @@
     </row>
     <row r="6" ht="15" customHeight="1" s="58">
       <c r="C6" s="82" t="n">
-        <v>46150.5</v>
+        <v>46120.5</v>
       </c>
       <c r="D6" s="82" t="n">
-        <v>46157.5</v>
+        <v>46127.5</v>
       </c>
       <c r="G6" s="52" t="inlineStr">
         <is>
@@ -2745,7 +2758,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="82" t="n">
-        <v>46143.41666666666</v>
+        <v>46113.41666666666</v>
       </c>
       <c r="D7" s="83" t="n"/>
       <c r="E7" s="52" t="inlineStr">
@@ -2907,7 +2920,7 @@
         </is>
       </c>
       <c r="G2" s="82" t="n">
-        <v>46145.41666666666</v>
+        <v>46115.41666666666</v>
       </c>
       <c r="H2" s="52" t="inlineStr">
         <is>
@@ -2943,7 +2956,7 @@
         </is>
       </c>
       <c r="G3" s="82" t="n">
-        <v>46145.41666666666</v>
+        <v>46115.41666666666</v>
       </c>
       <c r="H3" s="52" t="inlineStr">
         <is>
@@ -3622,7 +3635,7 @@
         </is>
       </c>
       <c r="E2" s="82" t="n">
-        <v>46145.4375</v>
+        <v>46115.4375</v>
       </c>
       <c r="F2" s="52" t="inlineStr">
         <is>
@@ -3655,7 +3668,7 @@
         </is>
       </c>
       <c r="E3" s="82" t="n">
-        <v>46145.4375</v>
+        <v>46115.4375</v>
       </c>
       <c r="F3" s="52" t="inlineStr">
         <is>
@@ -4066,7 +4079,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="82" t="n">
-        <v>46145.375</v>
+        <v>46115.375</v>
       </c>
       <c r="D2" s="52" t="inlineStr">
         <is>
@@ -4099,10 +4112,10 @@
         </is>
       </c>
       <c r="L2" s="82" t="n">
-        <v>46145.375</v>
+        <v>46115.375</v>
       </c>
       <c r="M2" s="82" t="n">
-        <v>46157.5</v>
+        <v>46127.5</v>
       </c>
       <c r="N2" s="52" t="n">
         <v>1</v>
@@ -4131,7 +4144,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="82" t="n">
-        <v>46145.375</v>
+        <v>46115.375</v>
       </c>
       <c r="D3" s="52" t="inlineStr">
         <is>
@@ -4164,10 +4177,10 @@
         </is>
       </c>
       <c r="L3" s="82" t="n">
-        <v>46145.375</v>
+        <v>46115.375</v>
       </c>
       <c r="M3" s="82" t="n">
-        <v>46157.5</v>
+        <v>46127.5</v>
       </c>
       <c r="N3" s="52" t="n">
         <v>1</v>
@@ -4196,7 +4209,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="82" t="n">
-        <v>46145.375</v>
+        <v>46115.375</v>
       </c>
       <c r="D4" s="52" t="inlineStr">
         <is>
@@ -4229,10 +4242,10 @@
         </is>
       </c>
       <c r="L4" s="82" t="n">
-        <v>46145.375</v>
+        <v>46115.375</v>
       </c>
       <c r="M4" s="82" t="n">
-        <v>46157.5</v>
+        <v>46127.5</v>
       </c>
       <c r="N4" s="52" t="n">
         <v>1</v>
@@ -4261,7 +4274,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="82" t="n">
-        <v>46145.375</v>
+        <v>46115.375</v>
       </c>
       <c r="D5" s="52" t="inlineStr">
         <is>
@@ -4294,7 +4307,7 @@
         </is>
       </c>
       <c r="L5" s="82" t="n">
-        <v>46145.375</v>
+        <v>46115.375</v>
       </c>
       <c r="M5" s="83" t="n"/>
       <c r="N5" s="52" t="n">
@@ -4584,7 +4597,7 @@
         </is>
       </c>
       <c r="G2" s="84" t="n">
-        <v>46145.35416666666</v>
+        <v>46115.35416666666</v>
       </c>
       <c r="H2" s="54" t="n"/>
     </row>
@@ -4616,7 +4629,7 @@
         </is>
       </c>
       <c r="G3" s="84" t="n">
-        <v>46145.35763888889</v>
+        <v>46115.35763888889</v>
       </c>
       <c r="H3" s="54" t="n"/>
     </row>
@@ -4648,7 +4661,7 @@
         </is>
       </c>
       <c r="G4" s="84" t="n">
-        <v>46145.35416666666</v>
+        <v>46115.35416666666</v>
       </c>
       <c r="H4" s="54" t="n"/>
     </row>
@@ -4680,7 +4693,7 @@
         </is>
       </c>
       <c r="G5" s="84" t="n">
-        <v>46145.35763888889</v>
+        <v>46115.35763888889</v>
       </c>
       <c r="H5" s="54" t="n"/>
     </row>
@@ -4712,7 +4725,7 @@
         </is>
       </c>
       <c r="G6" s="84" t="n">
-        <v>46145.35416666666</v>
+        <v>46115.35416666666</v>
       </c>
       <c r="H6" s="54" t="n"/>
     </row>
@@ -4744,7 +4757,7 @@
         </is>
       </c>
       <c r="G7" s="84" t="n">
-        <v>46145.35763888889</v>
+        <v>46115.35763888889</v>
       </c>
       <c r="H7" s="54" t="n"/>
     </row>
@@ -4875,7 +4888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A2:U252"/>
+  <dimension ref="A1:U252"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12.15" customWidth="1" style="52" min="1" max="1"/>
@@ -4889,6 +4902,7 @@
     <col width="14.57" customWidth="1" style="52" min="14" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="15" customHeight="1" s="58">
       <c r="D2" s="76" t="inlineStr">
         <is>

</xml_diff>